<commit_message>
changement de fiche synthèse et retrait de projet
</commit_message>
<xml_diff>
--- a/assets/documents/tableau_synthese.xlsx
+++ b/assets/documents/tableau_synthese.xlsx
@@ -118,7 +118,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -641,6 +641,34 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
@@ -1224,7 +1252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75"/>
   <cols>
     <col width="70.42578125" customWidth="1" style="1" min="1" max="1"/>
@@ -1741,80 +1769,7 @@
       <c r="H21" s="55" t="n"/>
     </row>
     <row r="22" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A22" s="63" t="inlineStr">
-        <is>
-          <t>Fondation.io - Landing Page (site vitrine)
-Technos : HTML, CSS
-Docs : Dépôt GitHub Fondation-io/landing-page</t>
-        </is>
-      </c>
-      <c r="B22" s="63" t="inlineStr">
-        <is>
-          <t>01/09/25 au 31/10/25</t>
-        </is>
-      </c>
-      <c r="C22" s="64" t="n"/>
-      <c r="D22" s="65" t="n"/>
-      <c r="E22" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F22" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G22" s="65" t="n"/>
-      <c r="H22" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A23" s="63" t="inlineStr">
-        <is>
-          <t>Fondation.io - fast-db-batch-search-client
-Client TypeScript pour API de recherche batch (fuzzy search, jointures, CI/CD)
-Technos : TypeScript, Node.js, API REST, GitHub Actions
-Docs : Dépôt GitHub Fondation-io/fast-db-batch-search-client | npm @fondation-io/fast-db-batch-search-client</t>
-        </is>
-      </c>
-      <c r="B23" s="63" t="inlineStr">
-        <is>
-          <t>01/11/25 au 31/01/26</t>
-        </is>
-      </c>
-      <c r="C23" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D23" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E23" s="66" t="n"/>
-      <c r="F23" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G23" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H23" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="70" customFormat="1" customHeight="1" s="2">
-      <c r="A24" s="72" t="inlineStr">
+      <c r="A22" s="72" t="inlineStr">
         <is>
           <t>Fondation.io - Comparateur d'IA Automatisé (Testing_Claude_code)
 Framework de benchmark de LLMs en parallèle, export JSON/CSV
@@ -1822,32 +1777,108 @@
 Docs : Dépôt privé entreprise</t>
         </is>
       </c>
-      <c r="B24" s="73" t="inlineStr">
+      <c r="B22" s="73" t="inlineStr">
         <is>
           <t>01/02/25 au 30/04/25</t>
         </is>
       </c>
-      <c r="C24" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C22" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G22" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="n"/>
+    </row>
+    <row r="23" ht="39.95" customFormat="1" customHeight="1" s="2">
+      <c r="A23" s="72" t="inlineStr">
+        <is>
+          <t>Fondation.io - Scanner de Flux RSS Intelligent (RSSScanner)
+Veille tech automatisée multi-sources, parseur OPML, déduplication
+Technos : Python, RSS, Data Parsing, Backend
+Docs : Dépôt privé entreprise</t>
+        </is>
+      </c>
+      <c r="B23" s="73" t="inlineStr">
+        <is>
+          <t>01/06/25 au 31/08/25</t>
+        </is>
+      </c>
+      <c r="C23" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="75" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="A24" s="72" t="n"/>
+      <c r="B24" s="73" t="n"/>
+      <c r="C24" s="74" t="n"/>
       <c r="D24" s="21" t="n"/>
       <c r="E24" s="21" t="n"/>
-      <c r="F24" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G24" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="F24" s="74" t="n"/>
+      <c r="G24" s="74" t="n"/>
       <c r="H24" s="22" t="n"/>
     </row>
     <row r="25" ht="70" customFormat="1" customHeight="1" s="2">
-      <c r="A25" s="72" t="inlineStr">
+      <c r="A25" s="72" t="n"/>
+      <c r="B25" s="73" t="n"/>
+      <c r="C25" s="74" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="21" t="n"/>
+      <c r="F25" s="21" t="n"/>
+      <c r="G25" s="21" t="n"/>
+      <c r="H25" s="75" t="n"/>
+    </row>
+    <row r="26" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="A26" s="13" t="n"/>
+      <c r="B26" s="54" t="n"/>
+      <c r="C26" s="54" t="n"/>
+      <c r="D26" s="54" t="n"/>
+      <c r="E26" s="54" t="n"/>
+      <c r="F26" s="54" t="n"/>
+      <c r="G26" s="54" t="n"/>
+      <c r="H26" s="55" t="n"/>
+    </row>
+    <row r="27" ht="18" customFormat="1" customHeight="1" s="2">
+      <c r="A27" s="13" t="n"/>
+    </row>
+    <row r="28" ht="39.95" customFormat="1" customHeight="1" s="2">
+      <c r="A28" s="32" t="inlineStr">
+        <is>
+          <t>Réalisations en milieu professionnel en cours de seconde année</t>
+        </is>
+      </c>
+      <c r="B28" s="54" t="n"/>
+      <c r="C28" s="54" t="n"/>
+      <c r="D28" s="54" t="n"/>
+      <c r="E28" s="54" t="n"/>
+      <c r="F28" s="54" t="n"/>
+      <c r="G28" s="54" t="n"/>
+      <c r="H28" s="55" t="n"/>
+    </row>
+    <row r="29" ht="30" customFormat="1" customHeight="1" s="2">
+      <c r="A29" s="72" t="inlineStr">
         <is>
           <t>Fondation.io - AgentSea
 Agents IA autonomes navigant sur le web (headless browsers, LLM-piloté)
@@ -1855,129 +1886,39 @@
 Docs : Dépôt privé entreprise</t>
         </is>
       </c>
-      <c r="B25" s="73" t="inlineStr">
+      <c r="B29" s="73" t="inlineStr">
         <is>
           <t>01/05/25 au 31/07/25</t>
         </is>
       </c>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E25" s="21" t="n"/>
-      <c r="F25" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G25" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H25" s="22" t="n"/>
-    </row>
-    <row r="26" ht="70" customFormat="1" customHeight="1" s="2">
-      <c r="A26" s="72" t="inlineStr">
-        <is>
-          <t>Fondation.io - Scanner de Flux RSS Intelligent (RSSScanner)
-Veille tech automatisée multi-sources, parseur OPML, déduplication
-Technos : Python, RSS, Data Parsing, Backend
-Docs : Dépôt privé entreprise</t>
-        </is>
-      </c>
-      <c r="B26" s="73" t="inlineStr">
-        <is>
-          <t>01/06/25 au 31/08/25</t>
-        </is>
-      </c>
-      <c r="C26" s="74" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="21" t="n"/>
-      <c r="F26" s="21" t="n"/>
-      <c r="G26" s="21" t="n"/>
-      <c r="H26" s="75" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customFormat="1" customHeight="1" s="2">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="54" t="n"/>
-      <c r="C27" s="54" t="n"/>
-      <c r="D27" s="54" t="n"/>
-      <c r="E27" s="54" t="n"/>
-      <c r="F27" s="54" t="n"/>
-      <c r="G27" s="54" t="n"/>
-      <c r="H27" s="55" t="n"/>
-    </row>
-    <row r="28" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A28" s="13" t="n"/>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="21" t="n"/>
-      <c r="D28" s="21" t="n"/>
-      <c r="E28" s="21" t="n"/>
-      <c r="F28" s="21" t="n"/>
-      <c r="G28" s="21" t="n"/>
-      <c r="H28" s="22" t="n"/>
-    </row>
-    <row r="29" ht="30" customFormat="1" customHeight="1" s="2">
-      <c r="A29" s="32" t="inlineStr">
-        <is>
-          <t>Réalisations en milieu professionnel en cours de seconde année</t>
-        </is>
-      </c>
-      <c r="B29" s="54" t="n"/>
-      <c r="C29" s="54" t="n"/>
-      <c r="D29" s="54" t="n"/>
-      <c r="E29" s="54" t="n"/>
-      <c r="F29" s="54" t="n"/>
-      <c r="G29" s="54" t="n"/>
-      <c r="H29" s="55" t="n"/>
-    </row>
-    <row r="30" ht="39.95" customFormat="1" customHeight="1" s="2">
-      <c r="A30" s="63" t="inlineStr">
-        <is>
-          <t>Fondation.io - Codex (fork openai/codex)
-Agent de code IA s'exécutant en terminal (contribution open source)
-Technos : Rust, IA générative, CLI
-Docs : Dépôt GitHub Fondation-io/codex</t>
-        </is>
-      </c>
-      <c r="B30" s="63" t="inlineStr">
-        <is>
-          <t>01/02/26 au 31/03/26</t>
-        </is>
-      </c>
-      <c r="C30" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D30" s="65" t="n"/>
-      <c r="E30" s="66" t="n"/>
-      <c r="F30" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G30" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H30" s="69" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E29" s="21" t="n"/>
+      <c r="F29" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G29" s="74" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="n"/>
+    </row>
+    <row r="30" ht="70" customFormat="1" customHeight="1" s="2">
+      <c r="A30" s="72" t="n"/>
+      <c r="B30" s="73" t="n"/>
+      <c r="C30" s="21" t="n"/>
+      <c r="D30" s="74" t="n"/>
+      <c r="E30" s="21" t="n"/>
+      <c r="F30" s="74" t="n"/>
+      <c r="G30" s="74" t="n"/>
+      <c r="H30" s="22" t="n"/>
     </row>
     <row r="31" ht="39.95" customFormat="1" customHeight="1" s="2">
       <c r="A31" s="13" t="n"/>
@@ -2020,48 +1961,38 @@
       <c r="H34" s="22" t="n"/>
     </row>
     <row r="35" ht="15" customFormat="1" customHeight="1" s="2">
-      <c r="A35" s="13" t="n"/>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="21" t="n"/>
-      <c r="E35" s="21" t="n"/>
-      <c r="F35" s="21" t="n"/>
-      <c r="G35" s="21" t="n"/>
-      <c r="H35" s="22" t="n"/>
+      <c r="A35" s="14" t="n"/>
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="23" t="n"/>
+      <c r="D35" s="23" t="n"/>
+      <c r="E35" s="23" t="n"/>
+      <c r="F35" s="23" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="24" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="24" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
+      <c r="A36" s="5" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A29:H29"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A27:H27"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A8:H8"/>

</xml_diff>